<commit_message>
feat(admin): add wide modal back buttons, drawer-to-modal filter sync, dynamic semester options, and dashboard-level report Excel download
</commit_message>
<xml_diff>
--- a/student_list passout 2028.xlsx
+++ b/student_list passout 2028.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:E250"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,6 +414,12 @@
       <c r="C2" t="str">
         <v>Enrollment No.</v>
       </c>
+      <c r="D2" t="str">
+        <v>Year</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Section</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -425,6 +431,12 @@
       <c r="C3" t="str">
         <v>12024002037042</v>
       </c>
+      <c r="D3" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -436,6 +448,12 @@
       <c r="C4" t="str">
         <v>12024002037046</v>
       </c>
+      <c r="D4" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -447,6 +465,12 @@
       <c r="C5" t="str">
         <v>12024002037011</v>
       </c>
+      <c r="D5" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -458,6 +482,12 @@
       <c r="C6" t="str">
         <v>12024002037056</v>
       </c>
+      <c r="D6" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -469,6 +499,12 @@
       <c r="C7" t="str">
         <v>12024002037024</v>
       </c>
+      <c r="D7" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -480,6 +516,12 @@
       <c r="C8" t="str">
         <v>12024002037053</v>
       </c>
+      <c r="D8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -491,6 +533,12 @@
       <c r="C9" t="str">
         <v>12024002037002</v>
       </c>
+      <c r="D9" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -502,6 +550,12 @@
       <c r="C10" t="str">
         <v>12024002037043</v>
       </c>
+      <c r="D10" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -513,6 +567,12 @@
       <c r="C11" t="str">
         <v>12024002037017</v>
       </c>
+      <c r="D11" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -524,6 +584,12 @@
       <c r="C12" t="str">
         <v>12024002037050</v>
       </c>
+      <c r="D12" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -535,6 +601,12 @@
       <c r="C13" t="str">
         <v>12024002037015</v>
       </c>
+      <c r="D13" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -546,6 +618,12 @@
       <c r="C14" t="str">
         <v>12024002037020</v>
       </c>
+      <c r="D14" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -557,6 +635,12 @@
       <c r="C15" t="str">
         <v>12024002037047</v>
       </c>
+      <c r="D15" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -568,6 +652,12 @@
       <c r="C16" t="str">
         <v>12024002037048</v>
       </c>
+      <c r="D16" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -579,6 +669,12 @@
       <c r="C17" t="str">
         <v>12024002037022</v>
       </c>
+      <c r="D17" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -590,6 +686,12 @@
       <c r="C18" t="str">
         <v>12024002037004</v>
       </c>
+      <c r="D18" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -601,6 +703,12 @@
       <c r="C19" t="str">
         <v>12024002037027</v>
       </c>
+      <c r="D19" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -612,6 +720,12 @@
       <c r="C20" t="str">
         <v>12024002037052</v>
       </c>
+      <c r="D20" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -623,6 +737,12 @@
       <c r="C21" t="str">
         <v>12024002037060</v>
       </c>
+      <c r="D21" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -634,6 +754,12 @@
       <c r="C22" t="str">
         <v>12024002037035</v>
       </c>
+      <c r="D22" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -645,6 +771,12 @@
       <c r="C23" t="str">
         <v>12024002037049</v>
       </c>
+      <c r="D23" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -656,6 +788,12 @@
       <c r="C24" t="str">
         <v>12024002037021</v>
       </c>
+      <c r="D24" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -667,6 +805,12 @@
       <c r="C25" t="str">
         <v>12024002037055</v>
       </c>
+      <c r="D25" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -678,6 +822,12 @@
       <c r="C26" t="str">
         <v>12024002037034</v>
       </c>
+      <c r="D26" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -689,6 +839,12 @@
       <c r="C27" t="str">
         <v>12024002037039</v>
       </c>
+      <c r="D27" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -700,6 +856,12 @@
       <c r="C28" t="str">
         <v>12024002037063</v>
       </c>
+      <c r="D28" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -711,6 +873,12 @@
       <c r="C29" t="str">
         <v>12024002037023</v>
       </c>
+      <c r="D29" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -722,6 +890,12 @@
       <c r="C30" t="str">
         <v>12024002037036</v>
       </c>
+      <c r="D30" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -733,6 +907,12 @@
       <c r="C31" t="str">
         <v>12024002037010</v>
       </c>
+      <c r="D31" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -744,6 +924,12 @@
       <c r="C32" t="str">
         <v>12024002037031</v>
       </c>
+      <c r="D32" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -755,6 +941,12 @@
       <c r="C33" t="str">
         <v>12024002037044</v>
       </c>
+      <c r="D33" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -766,6 +958,12 @@
       <c r="C34" t="str">
         <v>12024002037029</v>
       </c>
+      <c r="D34" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -777,6 +975,12 @@
       <c r="C35" t="str">
         <v>12024002037012</v>
       </c>
+      <c r="D35" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -788,6 +992,12 @@
       <c r="C36" t="str">
         <v>12024002037062</v>
       </c>
+      <c r="D36" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -799,6 +1009,12 @@
       <c r="C37" t="str">
         <v>12024002037058</v>
       </c>
+      <c r="D37" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -810,6 +1026,12 @@
       <c r="C38" t="str">
         <v>12024002037006</v>
       </c>
+      <c r="D38" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -821,6 +1043,12 @@
       <c r="C39" t="str">
         <v>12024002037005</v>
       </c>
+      <c r="D39" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -832,6 +1060,12 @@
       <c r="C40" t="str">
         <v>12024002037032</v>
       </c>
+      <c r="D40" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -843,6 +1077,12 @@
       <c r="C41" t="str">
         <v>12024002037008</v>
       </c>
+      <c r="D41" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -854,6 +1094,12 @@
       <c r="C42" t="str">
         <v>12024002037014</v>
       </c>
+      <c r="D42" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -865,6 +1111,12 @@
       <c r="C43" t="str">
         <v>12024002037045</v>
       </c>
+      <c r="D43" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -876,6 +1128,12 @@
       <c r="C44" t="str">
         <v>12024002037037</v>
       </c>
+      <c r="D44" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -887,6 +1145,12 @@
       <c r="C45" t="str">
         <v>12024002037041</v>
       </c>
+      <c r="D45" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -898,6 +1162,12 @@
       <c r="C46" t="str">
         <v>12024002037018</v>
       </c>
+      <c r="D46" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -909,6 +1179,12 @@
       <c r="C47" t="str">
         <v>12024002037003</v>
       </c>
+      <c r="D47" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -920,6 +1196,12 @@
       <c r="C48" t="str">
         <v>12024002037054</v>
       </c>
+      <c r="D48" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -931,6 +1213,12 @@
       <c r="C49" t="str">
         <v>12024002037016</v>
       </c>
+      <c r="D49" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -942,6 +1230,12 @@
       <c r="C50" t="str">
         <v>12024002037064</v>
       </c>
+      <c r="D50" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -953,6 +1247,12 @@
       <c r="C51" t="str">
         <v>12024002037028</v>
       </c>
+      <c r="D51" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -964,6 +1264,12 @@
       <c r="C52" t="str">
         <v>12024002037013</v>
       </c>
+      <c r="D52" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -975,6 +1281,12 @@
       <c r="C53" t="str">
         <v>12024002037040</v>
       </c>
+      <c r="D53" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -986,6 +1298,12 @@
       <c r="C54" t="str">
         <v>12024002037009</v>
       </c>
+      <c r="D54" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -997,6 +1315,12 @@
       <c r="C55" t="str">
         <v>12024002037030</v>
       </c>
+      <c r="D55" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -1008,6 +1332,12 @@
       <c r="C56" t="str">
         <v>12024002037025</v>
       </c>
+      <c r="D56" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -1019,6 +1349,12 @@
       <c r="C57" t="str">
         <v>12024002037026</v>
       </c>
+      <c r="D57" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -1030,6 +1366,12 @@
       <c r="C58" t="str">
         <v>12024002037038</v>
       </c>
+      <c r="D58" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -1041,6 +1383,12 @@
       <c r="C59" t="str">
         <v>12024002037001</v>
       </c>
+      <c r="D59" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -1052,6 +1400,12 @@
       <c r="C60" t="str">
         <v>12024002037019</v>
       </c>
+      <c r="D60" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -1063,6 +1417,12 @@
       <c r="C61" t="str">
         <v>12024002037057</v>
       </c>
+      <c r="D61" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -1074,6 +1434,12 @@
       <c r="C62" t="str">
         <v>12024002037061</v>
       </c>
+      <c r="D62" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -1085,6 +1451,12 @@
       <c r="C63" t="str">
         <v>12024002037033</v>
       </c>
+      <c r="D63" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -1096,10 +1468,3178 @@
       <c r="C64" t="str">
         <v>12024002037059</v>
       </c>
+      <c r="D64" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>1</v>
+      </c>
+      <c r="B65" t="str">
+        <v>ARGHADEEP MANDAL</v>
+      </c>
+      <c r="C65" t="str">
+        <v>120220002037001</v>
+      </c>
+      <c r="D65" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>2</v>
+      </c>
+      <c r="B66" t="str">
+        <v>PRANJAL GHOSH</v>
+      </c>
+      <c r="C66" t="str">
+        <v>120220002037002</v>
+      </c>
+      <c r="D66" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>3</v>
+      </c>
+      <c r="B67" t="str">
+        <v>SOMNATH SHAW</v>
+      </c>
+      <c r="C67" t="str">
+        <v>120220002037003</v>
+      </c>
+      <c r="D67" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>4</v>
+      </c>
+      <c r="B68" t="str">
+        <v>RIYA PANDA</v>
+      </c>
+      <c r="C68" t="str">
+        <v>120220002037004</v>
+      </c>
+      <c r="D68" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>5</v>
+      </c>
+      <c r="B69" t="str">
+        <v>BISWAJIT BISWAS</v>
+      </c>
+      <c r="C69" t="str">
+        <v>120220002037005</v>
+      </c>
+      <c r="D69" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>6</v>
+      </c>
+      <c r="B70" t="str">
+        <v>ISHITA ROY</v>
+      </c>
+      <c r="C70" t="str">
+        <v>120220002037006</v>
+      </c>
+      <c r="D70" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>7</v>
+      </c>
+      <c r="B71" t="str">
+        <v>ABHISHEK BARMAN</v>
+      </c>
+      <c r="C71" t="str">
+        <v>120220002037007</v>
+      </c>
+      <c r="D71" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>8</v>
+      </c>
+      <c r="B72" t="str">
+        <v>SAYANI MAJUMDER</v>
+      </c>
+      <c r="C72" t="str">
+        <v>120220002037008</v>
+      </c>
+      <c r="D72" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>9</v>
+      </c>
+      <c r="B73" t="str">
+        <v>MITALI KUMAR</v>
+      </c>
+      <c r="C73" t="str">
+        <v>120220002037009</v>
+      </c>
+      <c r="D73" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>10</v>
+      </c>
+      <c r="B74" t="str">
+        <v>BISWAJIT SAHA</v>
+      </c>
+      <c r="C74" t="str">
+        <v>120220002037010</v>
+      </c>
+      <c r="D74" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>11</v>
+      </c>
+      <c r="B75" t="str">
+        <v>BARSHA DEY</v>
+      </c>
+      <c r="C75" t="str">
+        <v>120220002037011</v>
+      </c>
+      <c r="D75" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>12</v>
+      </c>
+      <c r="B76" t="str">
+        <v>SHATABDI NATH</v>
+      </c>
+      <c r="C76" t="str">
+        <v>120220002037012</v>
+      </c>
+      <c r="D76" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>13</v>
+      </c>
+      <c r="B77" t="str">
+        <v>RACHANA PRAMANIK</v>
+      </c>
+      <c r="C77" t="str">
+        <v>120220002037013</v>
+      </c>
+      <c r="D77" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>14</v>
+      </c>
+      <c r="B78" t="str">
+        <v>RUPSA SARKAR</v>
+      </c>
+      <c r="C78" t="str">
+        <v>120220002037014</v>
+      </c>
+      <c r="D78" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>15</v>
+      </c>
+      <c r="B79" t="str">
+        <v>RUDRA SARKAR</v>
+      </c>
+      <c r="C79" t="str">
+        <v>120220002037015</v>
+      </c>
+      <c r="D79" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>16</v>
+      </c>
+      <c r="B80" t="str">
+        <v>PALLABI ADHIKARI</v>
+      </c>
+      <c r="C80" t="str">
+        <v>120220002037016</v>
+      </c>
+      <c r="D80" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>17</v>
+      </c>
+      <c r="B81" t="str">
+        <v>MADHUMITA GIRI</v>
+      </c>
+      <c r="C81" t="str">
+        <v>120220002037017</v>
+      </c>
+      <c r="D81" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>18</v>
+      </c>
+      <c r="B82" t="str">
+        <v>RUDRA ADHIKARI</v>
+      </c>
+      <c r="C82" t="str">
+        <v>120220002037018</v>
+      </c>
+      <c r="D82" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>19</v>
+      </c>
+      <c r="B83" t="str">
+        <v>KOUSHIK NASKAR</v>
+      </c>
+      <c r="C83" t="str">
+        <v>120220002037019</v>
+      </c>
+      <c r="D83" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>20</v>
+      </c>
+      <c r="B84" t="str">
+        <v>TANMOY MAJUMDER</v>
+      </c>
+      <c r="C84" t="str">
+        <v>120220002037020</v>
+      </c>
+      <c r="D84" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>21</v>
+      </c>
+      <c r="B85" t="str">
+        <v>SHATABDI SAMANTA</v>
+      </c>
+      <c r="C85" t="str">
+        <v>120220002037021</v>
+      </c>
+      <c r="D85" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>22</v>
+      </c>
+      <c r="B86" t="str">
+        <v>DEBADUTTA DEY</v>
+      </c>
+      <c r="C86" t="str">
+        <v>120220002037022</v>
+      </c>
+      <c r="D86" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>23</v>
+      </c>
+      <c r="B87" t="str">
+        <v>SAYANTAN MANDAL</v>
+      </c>
+      <c r="C87" t="str">
+        <v>120220002037023</v>
+      </c>
+      <c r="D87" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>24</v>
+      </c>
+      <c r="B88" t="str">
+        <v>DEBOJYOTI PATHAK</v>
+      </c>
+      <c r="C88" t="str">
+        <v>120220002037024</v>
+      </c>
+      <c r="D88" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>25</v>
+      </c>
+      <c r="B89" t="str">
+        <v>SUBHAM SARKAR</v>
+      </c>
+      <c r="C89" t="str">
+        <v>120220002037025</v>
+      </c>
+      <c r="D89" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>26</v>
+      </c>
+      <c r="B90" t="str">
+        <v>MD SAHIL SINGH</v>
+      </c>
+      <c r="C90" t="str">
+        <v>120220002037026</v>
+      </c>
+      <c r="D90" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>27</v>
+      </c>
+      <c r="B91" t="str">
+        <v>PARAMITA SEN</v>
+      </c>
+      <c r="C91" t="str">
+        <v>120220002037027</v>
+      </c>
+      <c r="D91" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>28</v>
+      </c>
+      <c r="B92" t="str">
+        <v>PRIYANKA BISWAS</v>
+      </c>
+      <c r="C92" t="str">
+        <v>120220002037028</v>
+      </c>
+      <c r="D92" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>29</v>
+      </c>
+      <c r="B93" t="str">
+        <v>ARNAB SEN</v>
+      </c>
+      <c r="C93" t="str">
+        <v>120220002037029</v>
+      </c>
+      <c r="D93" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>30</v>
+      </c>
+      <c r="B94" t="str">
+        <v>RUPSA HALDAR</v>
+      </c>
+      <c r="C94" t="str">
+        <v>120220002037030</v>
+      </c>
+      <c r="D94" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>31</v>
+      </c>
+      <c r="B95" t="str">
+        <v>RUDRA GIRI</v>
+      </c>
+      <c r="C95" t="str">
+        <v>120220002037031</v>
+      </c>
+      <c r="D95" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>32</v>
+      </c>
+      <c r="B96" t="str">
+        <v>SOUMYADEEP DAS</v>
+      </c>
+      <c r="C96" t="str">
+        <v>120220002037032</v>
+      </c>
+      <c r="D96" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>33</v>
+      </c>
+      <c r="B97" t="str">
+        <v>SUBHAM SINGH</v>
+      </c>
+      <c r="C97" t="str">
+        <v>120220002037033</v>
+      </c>
+      <c r="D97" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>34</v>
+      </c>
+      <c r="B98" t="str">
+        <v>MITALI GIRI</v>
+      </c>
+      <c r="C98" t="str">
+        <v>120220002037034</v>
+      </c>
+      <c r="D98" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>35</v>
+      </c>
+      <c r="B99" t="str">
+        <v>ANINDITA BANERJEE</v>
+      </c>
+      <c r="C99" t="str">
+        <v>120220002037035</v>
+      </c>
+      <c r="D99" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>36</v>
+      </c>
+      <c r="B100" t="str">
+        <v>PRANJAL PRAMANIK</v>
+      </c>
+      <c r="C100" t="str">
+        <v>120220002037036</v>
+      </c>
+      <c r="D100" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>37</v>
+      </c>
+      <c r="B101" t="str">
+        <v>TRISHA MONDAL</v>
+      </c>
+      <c r="C101" t="str">
+        <v>120220002037037</v>
+      </c>
+      <c r="D101" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>38</v>
+      </c>
+      <c r="B102" t="str">
+        <v>KUNAL NASKAR</v>
+      </c>
+      <c r="C102" t="str">
+        <v>120220002037038</v>
+      </c>
+      <c r="D102" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>39</v>
+      </c>
+      <c r="B103" t="str">
+        <v>MOUMITA KAR</v>
+      </c>
+      <c r="C103" t="str">
+        <v>120220002037039</v>
+      </c>
+      <c r="D103" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>40</v>
+      </c>
+      <c r="B104" t="str">
+        <v>AMIT ADHIKARI</v>
+      </c>
+      <c r="C104" t="str">
+        <v>120220002037040</v>
+      </c>
+      <c r="D104" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>41</v>
+      </c>
+      <c r="B105" t="str">
+        <v>MITALI ADHIKARI</v>
+      </c>
+      <c r="C105" t="str">
+        <v>120220002037041</v>
+      </c>
+      <c r="D105" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>42</v>
+      </c>
+      <c r="B106" t="str">
+        <v>RUDRA HALDAR</v>
+      </c>
+      <c r="C106" t="str">
+        <v>120220002037042</v>
+      </c>
+      <c r="D106" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>43</v>
+      </c>
+      <c r="B107" t="str">
+        <v>ANINDITA PAL</v>
+      </c>
+      <c r="C107" t="str">
+        <v>120220002037043</v>
+      </c>
+      <c r="D107" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>44</v>
+      </c>
+      <c r="B108" t="str">
+        <v>DEBADUTTA BARMAN</v>
+      </c>
+      <c r="C108" t="str">
+        <v>120220002037044</v>
+      </c>
+      <c r="D108" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>45</v>
+      </c>
+      <c r="B109" t="str">
+        <v>ANKITA PATHAK</v>
+      </c>
+      <c r="C109" t="str">
+        <v>120220002037045</v>
+      </c>
+      <c r="D109" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>46</v>
+      </c>
+      <c r="B110" t="str">
+        <v>NILADRI CHAKRABORTY</v>
+      </c>
+      <c r="C110" t="str">
+        <v>120220002037046</v>
+      </c>
+      <c r="D110" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>47</v>
+      </c>
+      <c r="B111" t="str">
+        <v>TANUSHREE SARKAR</v>
+      </c>
+      <c r="C111" t="str">
+        <v>120220002037047</v>
+      </c>
+      <c r="D111" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>48</v>
+      </c>
+      <c r="B112" t="str">
+        <v>DEBARATI MANDAL</v>
+      </c>
+      <c r="C112" t="str">
+        <v>120220002037048</v>
+      </c>
+      <c r="D112" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>49</v>
+      </c>
+      <c r="B113" t="str">
+        <v>MOUMITA GIRI</v>
+      </c>
+      <c r="C113" t="str">
+        <v>120220002037049</v>
+      </c>
+      <c r="D113" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>50</v>
+      </c>
+      <c r="B114" t="str">
+        <v>PRANJAL BARMAN</v>
+      </c>
+      <c r="C114" t="str">
+        <v>120220002037050</v>
+      </c>
+      <c r="D114" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>51</v>
+      </c>
+      <c r="B115" t="str">
+        <v>ANANYA BARMAN</v>
+      </c>
+      <c r="C115" t="str">
+        <v>120220002037051</v>
+      </c>
+      <c r="D115" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>52</v>
+      </c>
+      <c r="B116" t="str">
+        <v>AMIT SEN</v>
+      </c>
+      <c r="C116" t="str">
+        <v>120220002037052</v>
+      </c>
+      <c r="D116" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>53</v>
+      </c>
+      <c r="B117" t="str">
+        <v>BISWAJIT DEY</v>
+      </c>
+      <c r="C117" t="str">
+        <v>120220002037053</v>
+      </c>
+      <c r="D117" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>54</v>
+      </c>
+      <c r="B118" t="str">
+        <v>SOURAV MONDAL</v>
+      </c>
+      <c r="C118" t="str">
+        <v>120220002037054</v>
+      </c>
+      <c r="D118" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>55</v>
+      </c>
+      <c r="B119" t="str">
+        <v>ABIR SAMANTA</v>
+      </c>
+      <c r="C119" t="str">
+        <v>120220002037055</v>
+      </c>
+      <c r="D119" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>56</v>
+      </c>
+      <c r="B120" t="str">
+        <v>MITALI SHAW</v>
+      </c>
+      <c r="C120" t="str">
+        <v>120220002037056</v>
+      </c>
+      <c r="D120" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>57</v>
+      </c>
+      <c r="B121" t="str">
+        <v>SNEHASISH CHAKRABORTY</v>
+      </c>
+      <c r="C121" t="str">
+        <v>120220002037057</v>
+      </c>
+      <c r="D121" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>58</v>
+      </c>
+      <c r="B122" t="str">
+        <v>PALLABI GHOSH</v>
+      </c>
+      <c r="C122" t="str">
+        <v>120220002037058</v>
+      </c>
+      <c r="D122" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>59</v>
+      </c>
+      <c r="B123" t="str">
+        <v>PALLABI NATH</v>
+      </c>
+      <c r="C123" t="str">
+        <v>120220002037059</v>
+      </c>
+      <c r="D123" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>60</v>
+      </c>
+      <c r="B124" t="str">
+        <v>RAHUL ROY</v>
+      </c>
+      <c r="C124" t="str">
+        <v>120220002037060</v>
+      </c>
+      <c r="D124" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>61</v>
+      </c>
+      <c r="B125" t="str">
+        <v>SAYANTAN ADHIKARI</v>
+      </c>
+      <c r="C125" t="str">
+        <v>120220002037061</v>
+      </c>
+      <c r="D125" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>62</v>
+      </c>
+      <c r="B126" t="str">
+        <v>SUPRIYA SHAW</v>
+      </c>
+      <c r="C126" t="str">
+        <v>120220002037062</v>
+      </c>
+      <c r="D126" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>1</v>
+      </c>
+      <c r="B127" t="str">
+        <v>PRIYANKA MANDAL</v>
+      </c>
+      <c r="C127" t="str">
+        <v>120230002037001</v>
+      </c>
+      <c r="D127" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>2</v>
+      </c>
+      <c r="B128" t="str">
+        <v>SAGNIK MANDAL</v>
+      </c>
+      <c r="C128" t="str">
+        <v>120230002037002</v>
+      </c>
+      <c r="D128" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>3</v>
+      </c>
+      <c r="B129" t="str">
+        <v>NABANITA SARKAR</v>
+      </c>
+      <c r="C129" t="str">
+        <v>120230002037003</v>
+      </c>
+      <c r="D129" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>4</v>
+      </c>
+      <c r="B130" t="str">
+        <v>ARITRA DEY</v>
+      </c>
+      <c r="C130" t="str">
+        <v>120230002037004</v>
+      </c>
+      <c r="D130" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E130" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>5</v>
+      </c>
+      <c r="B131" t="str">
+        <v>SAYANI GIRI</v>
+      </c>
+      <c r="C131" t="str">
+        <v>120230002037005</v>
+      </c>
+      <c r="D131" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E131" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>6</v>
+      </c>
+      <c r="B132" t="str">
+        <v>MOUMITA BANERJEE</v>
+      </c>
+      <c r="C132" t="str">
+        <v>120230002037006</v>
+      </c>
+      <c r="D132" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E132" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>7</v>
+      </c>
+      <c r="B133" t="str">
+        <v>ANANYA PATHAK</v>
+      </c>
+      <c r="C133" t="str">
+        <v>120230002037007</v>
+      </c>
+      <c r="D133" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>8</v>
+      </c>
+      <c r="B134" t="str">
+        <v>PRIYA NASKAR</v>
+      </c>
+      <c r="C134" t="str">
+        <v>120230002037008</v>
+      </c>
+      <c r="D134" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>9</v>
+      </c>
+      <c r="B135" t="str">
+        <v>SAYANTANI KUMAR</v>
+      </c>
+      <c r="C135" t="str">
+        <v>120230002037009</v>
+      </c>
+      <c r="D135" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E135" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>10</v>
+      </c>
+      <c r="B136" t="str">
+        <v>SHREYA BISWAS</v>
+      </c>
+      <c r="C136" t="str">
+        <v>120230002037010</v>
+      </c>
+      <c r="D136" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>11</v>
+      </c>
+      <c r="B137" t="str">
+        <v>ARITRA PRAMANIK</v>
+      </c>
+      <c r="C137" t="str">
+        <v>120230002037011</v>
+      </c>
+      <c r="D137" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>12</v>
+      </c>
+      <c r="B138" t="str">
+        <v>DEBARATI KAR</v>
+      </c>
+      <c r="C138" t="str">
+        <v>120230002037012</v>
+      </c>
+      <c r="D138" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <v>13</v>
+      </c>
+      <c r="B139" t="str">
+        <v>TANMOY HALDAR</v>
+      </c>
+      <c r="C139" t="str">
+        <v>120230002037013</v>
+      </c>
+      <c r="D139" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>14</v>
+      </c>
+      <c r="B140" t="str">
+        <v>INDRANIL MONDAL</v>
+      </c>
+      <c r="C140" t="str">
+        <v>120230002037014</v>
+      </c>
+      <c r="D140" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E140" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>15</v>
+      </c>
+      <c r="B141" t="str">
+        <v>PALLABI DUTTA</v>
+      </c>
+      <c r="C141" t="str">
+        <v>120230002037015</v>
+      </c>
+      <c r="D141" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>16</v>
+      </c>
+      <c r="B142" t="str">
+        <v>PRIYANKA MAITY</v>
+      </c>
+      <c r="C142" t="str">
+        <v>120230002037016</v>
+      </c>
+      <c r="D142" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <v>17</v>
+      </c>
+      <c r="B143" t="str">
+        <v>SOURAV MAJUMDER</v>
+      </c>
+      <c r="C143" t="str">
+        <v>120230002037017</v>
+      </c>
+      <c r="D143" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <v>18</v>
+      </c>
+      <c r="B144" t="str">
+        <v>KOUSHIK DUTTA</v>
+      </c>
+      <c r="C144" t="str">
+        <v>120230002037018</v>
+      </c>
+      <c r="D144" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E144" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>19</v>
+      </c>
+      <c r="B145" t="str">
+        <v>AMIT ROY</v>
+      </c>
+      <c r="C145" t="str">
+        <v>120230002037019</v>
+      </c>
+      <c r="D145" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E145" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>20</v>
+      </c>
+      <c r="B146" t="str">
+        <v>DEBALINA PRAMANIK</v>
+      </c>
+      <c r="C146" t="str">
+        <v>120230002037020</v>
+      </c>
+      <c r="D146" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E146" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>21</v>
+      </c>
+      <c r="B147" t="str">
+        <v>DEBOJYOTI DUTTA</v>
+      </c>
+      <c r="C147" t="str">
+        <v>120230002037021</v>
+      </c>
+      <c r="D147" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E147" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>22</v>
+      </c>
+      <c r="B148" t="str">
+        <v>PRIYANKA NATH</v>
+      </c>
+      <c r="C148" t="str">
+        <v>120230002037022</v>
+      </c>
+      <c r="D148" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>23</v>
+      </c>
+      <c r="B149" t="str">
+        <v>RIYA PATHAK</v>
+      </c>
+      <c r="C149" t="str">
+        <v>120230002037023</v>
+      </c>
+      <c r="D149" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>24</v>
+      </c>
+      <c r="B150" t="str">
+        <v>TRISHA ROY</v>
+      </c>
+      <c r="C150" t="str">
+        <v>120230002037024</v>
+      </c>
+      <c r="D150" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E150" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>25</v>
+      </c>
+      <c r="B151" t="str">
+        <v>DEBADUTTA DUTTA</v>
+      </c>
+      <c r="C151" t="str">
+        <v>120230002037025</v>
+      </c>
+      <c r="D151" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E151" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>26</v>
+      </c>
+      <c r="B152" t="str">
+        <v>ISHITA SINGH</v>
+      </c>
+      <c r="C152" t="str">
+        <v>120230002037026</v>
+      </c>
+      <c r="D152" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E152" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>27</v>
+      </c>
+      <c r="B153" t="str">
+        <v>SUPRIYA SAHA</v>
+      </c>
+      <c r="C153" t="str">
+        <v>120230002037027</v>
+      </c>
+      <c r="D153" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E153" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>28</v>
+      </c>
+      <c r="B154" t="str">
+        <v>SAGNIK SARKAR</v>
+      </c>
+      <c r="C154" t="str">
+        <v>120230002037028</v>
+      </c>
+      <c r="D154" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E154" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <v>29</v>
+      </c>
+      <c r="B155" t="str">
+        <v>SAYANTANI BARMAN</v>
+      </c>
+      <c r="C155" t="str">
+        <v>120230002037029</v>
+      </c>
+      <c r="D155" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E155" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <v>30</v>
+      </c>
+      <c r="B156" t="str">
+        <v>MITALI MAJUMDER</v>
+      </c>
+      <c r="C156" t="str">
+        <v>120230002037030</v>
+      </c>
+      <c r="D156" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E156" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <v>31</v>
+      </c>
+      <c r="B157" t="str">
+        <v>RAHUL DEY</v>
+      </c>
+      <c r="C157" t="str">
+        <v>120230002037031</v>
+      </c>
+      <c r="D157" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E157" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <v>32</v>
+      </c>
+      <c r="B158" t="str">
+        <v>PALLABI PANDA</v>
+      </c>
+      <c r="C158" t="str">
+        <v>120230002037032</v>
+      </c>
+      <c r="D158" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <v>33</v>
+      </c>
+      <c r="B159" t="str">
+        <v>AYAN PANDA</v>
+      </c>
+      <c r="C159" t="str">
+        <v>120230002037033</v>
+      </c>
+      <c r="D159" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E159" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>34</v>
+      </c>
+      <c r="B160" t="str">
+        <v>SOUVIK SAHA</v>
+      </c>
+      <c r="C160" t="str">
+        <v>120230002037034</v>
+      </c>
+      <c r="D160" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E160" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>35</v>
+      </c>
+      <c r="B161" t="str">
+        <v>ANKITA MONDAL</v>
+      </c>
+      <c r="C161" t="str">
+        <v>120230002037035</v>
+      </c>
+      <c r="D161" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E161" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>36</v>
+      </c>
+      <c r="B162" t="str">
+        <v>ARITRA NASKAR</v>
+      </c>
+      <c r="C162" t="str">
+        <v>120230002037036</v>
+      </c>
+      <c r="D162" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E162" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>37</v>
+      </c>
+      <c r="B163" t="str">
+        <v>SAYAN NASKAR</v>
+      </c>
+      <c r="C163" t="str">
+        <v>120230002037037</v>
+      </c>
+      <c r="D163" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E163" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>38</v>
+      </c>
+      <c r="B164" t="str">
+        <v>SOUVIK KAR</v>
+      </c>
+      <c r="C164" t="str">
+        <v>120230002037038</v>
+      </c>
+      <c r="D164" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E164" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165">
+        <v>39</v>
+      </c>
+      <c r="B165" t="str">
+        <v>SOUMYADEEP ADHIKARI</v>
+      </c>
+      <c r="C165" t="str">
+        <v>120230002037039</v>
+      </c>
+      <c r="D165" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E165" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>40</v>
+      </c>
+      <c r="B166" t="str">
+        <v>DEBOJYOTI SINGH</v>
+      </c>
+      <c r="C166" t="str">
+        <v>120230002037040</v>
+      </c>
+      <c r="D166" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E166" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>41</v>
+      </c>
+      <c r="B167" t="str">
+        <v>BARSHA PRAMANIK</v>
+      </c>
+      <c r="C167" t="str">
+        <v>120230002037041</v>
+      </c>
+      <c r="D167" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E167" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>42</v>
+      </c>
+      <c r="B168" t="str">
+        <v>ANKITA GHOSH</v>
+      </c>
+      <c r="C168" t="str">
+        <v>120230002037042</v>
+      </c>
+      <c r="D168" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E168" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>43</v>
+      </c>
+      <c r="B169" t="str">
+        <v>SHATABDI ADHIKARI</v>
+      </c>
+      <c r="C169" t="str">
+        <v>120230002037043</v>
+      </c>
+      <c r="D169" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E169" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>44</v>
+      </c>
+      <c r="B170" t="str">
+        <v>TRISHA PANDA</v>
+      </c>
+      <c r="C170" t="str">
+        <v>120230002037044</v>
+      </c>
+      <c r="D170" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E170" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>45</v>
+      </c>
+      <c r="B171" t="str">
+        <v>PALLABI SAHA</v>
+      </c>
+      <c r="C171" t="str">
+        <v>120230002037045</v>
+      </c>
+      <c r="D171" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E171" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>46</v>
+      </c>
+      <c r="B172" t="str">
+        <v>TANUSHREE GIRI</v>
+      </c>
+      <c r="C172" t="str">
+        <v>120230002037046</v>
+      </c>
+      <c r="D172" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E172" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>47</v>
+      </c>
+      <c r="B173" t="str">
+        <v>INDRANIL SARKAR</v>
+      </c>
+      <c r="C173" t="str">
+        <v>120230002037047</v>
+      </c>
+      <c r="D173" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E173" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>48</v>
+      </c>
+      <c r="B174" t="str">
+        <v>PARAMITA PAL</v>
+      </c>
+      <c r="C174" t="str">
+        <v>120230002037048</v>
+      </c>
+      <c r="D174" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E174" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>49</v>
+      </c>
+      <c r="B175" t="str">
+        <v>ISHITA KAR</v>
+      </c>
+      <c r="C175" t="str">
+        <v>120230002037049</v>
+      </c>
+      <c r="D175" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E175" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>50</v>
+      </c>
+      <c r="B176" t="str">
+        <v>PALLABI PATHAK</v>
+      </c>
+      <c r="C176" t="str">
+        <v>120230002037050</v>
+      </c>
+      <c r="D176" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>51</v>
+      </c>
+      <c r="B177" t="str">
+        <v>ABIR ROY</v>
+      </c>
+      <c r="C177" t="str">
+        <v>120230002037051</v>
+      </c>
+      <c r="D177" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>52</v>
+      </c>
+      <c r="B178" t="str">
+        <v>INDRANIL PANDA</v>
+      </c>
+      <c r="C178" t="str">
+        <v>120230002037052</v>
+      </c>
+      <c r="D178" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>53</v>
+      </c>
+      <c r="B179" t="str">
+        <v>SOUMYADEEP PATHAK</v>
+      </c>
+      <c r="C179" t="str">
+        <v>120230002037053</v>
+      </c>
+      <c r="D179" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>54</v>
+      </c>
+      <c r="B180" t="str">
+        <v>MADHUMITA MONDAL</v>
+      </c>
+      <c r="C180" t="str">
+        <v>120230002037054</v>
+      </c>
+      <c r="D180" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E180" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>55</v>
+      </c>
+      <c r="B181" t="str">
+        <v>DEBOJYOTI PRAMANIK</v>
+      </c>
+      <c r="C181" t="str">
+        <v>120230002037055</v>
+      </c>
+      <c r="D181" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E181" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>56</v>
+      </c>
+      <c r="B182" t="str">
+        <v>SAGNIK SHAW</v>
+      </c>
+      <c r="C182" t="str">
+        <v>120230002037056</v>
+      </c>
+      <c r="D182" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>57</v>
+      </c>
+      <c r="B183" t="str">
+        <v>ABIR MANDAL</v>
+      </c>
+      <c r="C183" t="str">
+        <v>120230002037057</v>
+      </c>
+      <c r="D183" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>58</v>
+      </c>
+      <c r="B184" t="str">
+        <v>MOUMITA NASKAR</v>
+      </c>
+      <c r="C184" t="str">
+        <v>120230002037058</v>
+      </c>
+      <c r="D184" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185">
+        <v>59</v>
+      </c>
+      <c r="B185" t="str">
+        <v>SUPRIYA DEY</v>
+      </c>
+      <c r="C185" t="str">
+        <v>120230002037059</v>
+      </c>
+      <c r="D185" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186">
+        <v>60</v>
+      </c>
+      <c r="B186" t="str">
+        <v>ABHISHEK PATHAK</v>
+      </c>
+      <c r="C186" t="str">
+        <v>120230002037060</v>
+      </c>
+      <c r="D186" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187">
+        <v>61</v>
+      </c>
+      <c r="B187" t="str">
+        <v>DEBOJYOTI PAL</v>
+      </c>
+      <c r="C187" t="str">
+        <v>120230002037061</v>
+      </c>
+      <c r="D187" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188">
+        <v>62</v>
+      </c>
+      <c r="B188" t="str">
+        <v>ARNAB DAS</v>
+      </c>
+      <c r="C188" t="str">
+        <v>120230002037062</v>
+      </c>
+      <c r="D188" t="str">
+        <v>3rd Year</v>
+      </c>
+      <c r="E188" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189">
+        <v>1</v>
+      </c>
+      <c r="B189" t="str">
+        <v>NILADRI MONDAL</v>
+      </c>
+      <c r="C189" t="str">
+        <v>120250002037001</v>
+      </c>
+      <c r="D189" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190">
+        <v>2</v>
+      </c>
+      <c r="B190" t="str">
+        <v>SOURAV ADHIKARI</v>
+      </c>
+      <c r="C190" t="str">
+        <v>120250002037002</v>
+      </c>
+      <c r="D190" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E190" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191">
+        <v>3</v>
+      </c>
+      <c r="B191" t="str">
+        <v>ISHITA DUTTA</v>
+      </c>
+      <c r="C191" t="str">
+        <v>120250002037003</v>
+      </c>
+      <c r="D191" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E191" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192">
+        <v>4</v>
+      </c>
+      <c r="B192" t="str">
+        <v>SOMNATH SARKAR</v>
+      </c>
+      <c r="C192" t="str">
+        <v>120250002037004</v>
+      </c>
+      <c r="D192" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193">
+        <v>5</v>
+      </c>
+      <c r="B193" t="str">
+        <v>BISWAROOP MONDAL</v>
+      </c>
+      <c r="C193" t="str">
+        <v>120250002037005</v>
+      </c>
+      <c r="D193" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>6</v>
+      </c>
+      <c r="B194" t="str">
+        <v>SUSHMITA ADHIKARI</v>
+      </c>
+      <c r="C194" t="str">
+        <v>120250002037006</v>
+      </c>
+      <c r="D194" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>7</v>
+      </c>
+      <c r="B195" t="str">
+        <v>TANMOY GIRI</v>
+      </c>
+      <c r="C195" t="str">
+        <v>120250002037007</v>
+      </c>
+      <c r="D195" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>8</v>
+      </c>
+      <c r="B196" t="str">
+        <v>SAYANTAN MAJUMDER</v>
+      </c>
+      <c r="C196" t="str">
+        <v>120250002037008</v>
+      </c>
+      <c r="D196" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>9</v>
+      </c>
+      <c r="B197" t="str">
+        <v>PARAMITA GHOSH</v>
+      </c>
+      <c r="C197" t="str">
+        <v>120250002037009</v>
+      </c>
+      <c r="D197" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E197" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>10</v>
+      </c>
+      <c r="B198" t="str">
+        <v>SOURAV ROY</v>
+      </c>
+      <c r="C198" t="str">
+        <v>120250002037010</v>
+      </c>
+      <c r="D198" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E198" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>11</v>
+      </c>
+      <c r="B199" t="str">
+        <v>ABHISHEK DUTTA</v>
+      </c>
+      <c r="C199" t="str">
+        <v>120250002037011</v>
+      </c>
+      <c r="D199" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E199" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>12</v>
+      </c>
+      <c r="B200" t="str">
+        <v>DEBADUTTA SEN</v>
+      </c>
+      <c r="C200" t="str">
+        <v>120250002037012</v>
+      </c>
+      <c r="D200" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E200" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>13</v>
+      </c>
+      <c r="B201" t="str">
+        <v>SOURAV GIRI</v>
+      </c>
+      <c r="C201" t="str">
+        <v>120250002037013</v>
+      </c>
+      <c r="D201" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202">
+        <v>14</v>
+      </c>
+      <c r="B202" t="str">
+        <v>TANUSHREE KUMAR</v>
+      </c>
+      <c r="C202" t="str">
+        <v>120250002037014</v>
+      </c>
+      <c r="D202" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203">
+        <v>15</v>
+      </c>
+      <c r="B203" t="str">
+        <v>BARSHA KUMAR</v>
+      </c>
+      <c r="C203" t="str">
+        <v>120250002037015</v>
+      </c>
+      <c r="D203" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204">
+        <v>16</v>
+      </c>
+      <c r="B204" t="str">
+        <v>SAGNIK NASKAR</v>
+      </c>
+      <c r="C204" t="str">
+        <v>120250002037016</v>
+      </c>
+      <c r="D204" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205">
+        <v>17</v>
+      </c>
+      <c r="B205" t="str">
+        <v>SOMNATH KAR</v>
+      </c>
+      <c r="C205" t="str">
+        <v>120250002037017</v>
+      </c>
+      <c r="D205" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206">
+        <v>18</v>
+      </c>
+      <c r="B206" t="str">
+        <v>KOUSHIK BANERJEE</v>
+      </c>
+      <c r="C206" t="str">
+        <v>120250002037018</v>
+      </c>
+      <c r="D206" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207">
+        <v>19</v>
+      </c>
+      <c r="B207" t="str">
+        <v>SNEHASISH PATHAK</v>
+      </c>
+      <c r="C207" t="str">
+        <v>120250002037019</v>
+      </c>
+      <c r="D207" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208">
+        <v>20</v>
+      </c>
+      <c r="B208" t="str">
+        <v>AMIT MANDAL</v>
+      </c>
+      <c r="C208" t="str">
+        <v>120250002037020</v>
+      </c>
+      <c r="D208" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209">
+        <v>21</v>
+      </c>
+      <c r="B209" t="str">
+        <v>SNEHASISH PAL</v>
+      </c>
+      <c r="C209" t="str">
+        <v>120250002037021</v>
+      </c>
+      <c r="D209" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210">
+        <v>22</v>
+      </c>
+      <c r="B210" t="str">
+        <v>RITWIK NASKAR</v>
+      </c>
+      <c r="C210" t="str">
+        <v>120250002037022</v>
+      </c>
+      <c r="D210" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211">
+        <v>23</v>
+      </c>
+      <c r="B211" t="str">
+        <v>TRISHA BANERJEE</v>
+      </c>
+      <c r="C211" t="str">
+        <v>120250002037023</v>
+      </c>
+      <c r="D211" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212">
+        <v>24</v>
+      </c>
+      <c r="B212" t="str">
+        <v>RAJDEEP SAHA</v>
+      </c>
+      <c r="C212" t="str">
+        <v>120250002037024</v>
+      </c>
+      <c r="D212" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213">
+        <v>25</v>
+      </c>
+      <c r="B213" t="str">
+        <v>ANINDITA MAITY</v>
+      </c>
+      <c r="C213" t="str">
+        <v>120250002037025</v>
+      </c>
+      <c r="D213" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214">
+        <v>26</v>
+      </c>
+      <c r="B214" t="str">
+        <v>ANKITA ROY</v>
+      </c>
+      <c r="C214" t="str">
+        <v>120250002037026</v>
+      </c>
+      <c r="D214" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215">
+        <v>27</v>
+      </c>
+      <c r="B215" t="str">
+        <v>ARNAB MONDAL</v>
+      </c>
+      <c r="C215" t="str">
+        <v>120250002037027</v>
+      </c>
+      <c r="D215" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216">
+        <v>28</v>
+      </c>
+      <c r="B216" t="str">
+        <v>SAYAN PATHAK</v>
+      </c>
+      <c r="C216" t="str">
+        <v>120250002037028</v>
+      </c>
+      <c r="D216" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217">
+        <v>29</v>
+      </c>
+      <c r="B217" t="str">
+        <v>SAYAN SEN</v>
+      </c>
+      <c r="C217" t="str">
+        <v>120250002037029</v>
+      </c>
+      <c r="D217" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218">
+        <v>30</v>
+      </c>
+      <c r="B218" t="str">
+        <v>RUDRA PANDA</v>
+      </c>
+      <c r="C218" t="str">
+        <v>120250002037030</v>
+      </c>
+      <c r="D218" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219">
+        <v>31</v>
+      </c>
+      <c r="B219" t="str">
+        <v>RIYA ADHIKARI</v>
+      </c>
+      <c r="C219" t="str">
+        <v>120250002037031</v>
+      </c>
+      <c r="D219" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220">
+        <v>32</v>
+      </c>
+      <c r="B220" t="str">
+        <v>RUPSA GIRI</v>
+      </c>
+      <c r="C220" t="str">
+        <v>120250002037032</v>
+      </c>
+      <c r="D220" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221">
+        <v>33</v>
+      </c>
+      <c r="B221" t="str">
+        <v>SUBHAM BARMAN</v>
+      </c>
+      <c r="C221" t="str">
+        <v>120250002037033</v>
+      </c>
+      <c r="D221" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E221" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222">
+        <v>34</v>
+      </c>
+      <c r="B222" t="str">
+        <v>ARNAB ROY</v>
+      </c>
+      <c r="C222" t="str">
+        <v>120250002037034</v>
+      </c>
+      <c r="D222" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223">
+        <v>35</v>
+      </c>
+      <c r="B223" t="str">
+        <v>MADHUMITA CHAKRABORTY</v>
+      </c>
+      <c r="C223" t="str">
+        <v>120250002037035</v>
+      </c>
+      <c r="D223" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E223" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224">
+        <v>36</v>
+      </c>
+      <c r="B224" t="str">
+        <v>ARGHADEEP PRAMANIK</v>
+      </c>
+      <c r="C224" t="str">
+        <v>120250002037036</v>
+      </c>
+      <c r="D224" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225">
+        <v>37</v>
+      </c>
+      <c r="B225" t="str">
+        <v>SOUMEN NATH</v>
+      </c>
+      <c r="C225" t="str">
+        <v>120250002037037</v>
+      </c>
+      <c r="D225" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E225" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226">
+        <v>38</v>
+      </c>
+      <c r="B226" t="str">
+        <v>SOUMYADEEP SAMANTA</v>
+      </c>
+      <c r="C226" t="str">
+        <v>120250002037038</v>
+      </c>
+      <c r="D226" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227">
+        <v>39</v>
+      </c>
+      <c r="B227" t="str">
+        <v>RAHUL SAHA</v>
+      </c>
+      <c r="C227" t="str">
+        <v>120250002037039</v>
+      </c>
+      <c r="D227" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228">
+        <v>40</v>
+      </c>
+      <c r="B228" t="str">
+        <v>DEBALINA ROY</v>
+      </c>
+      <c r="C228" t="str">
+        <v>120250002037040</v>
+      </c>
+      <c r="D228" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229">
+        <v>41</v>
+      </c>
+      <c r="B229" t="str">
+        <v>RIYA SINGH</v>
+      </c>
+      <c r="C229" t="str">
+        <v>120250002037041</v>
+      </c>
+      <c r="D229" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230">
+        <v>42</v>
+      </c>
+      <c r="B230" t="str">
+        <v>SOMNATH MANDAL</v>
+      </c>
+      <c r="C230" t="str">
+        <v>120250002037042</v>
+      </c>
+      <c r="D230" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E230" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231">
+        <v>43</v>
+      </c>
+      <c r="B231" t="str">
+        <v>KUNAL ROY</v>
+      </c>
+      <c r="C231" t="str">
+        <v>120250002037043</v>
+      </c>
+      <c r="D231" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E231" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232">
+        <v>44</v>
+      </c>
+      <c r="B232" t="str">
+        <v>BIDISHA DUTTA</v>
+      </c>
+      <c r="C232" t="str">
+        <v>120250002037044</v>
+      </c>
+      <c r="D232" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E232" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233">
+        <v>45</v>
+      </c>
+      <c r="B233" t="str">
+        <v>SOUMYADEEP MONDAL</v>
+      </c>
+      <c r="C233" t="str">
+        <v>120250002037045</v>
+      </c>
+      <c r="D233" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234">
+        <v>46</v>
+      </c>
+      <c r="B234" t="str">
+        <v>ARNAB BANERJEE</v>
+      </c>
+      <c r="C234" t="str">
+        <v>120250002037046</v>
+      </c>
+      <c r="D234" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E234" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235">
+        <v>47</v>
+      </c>
+      <c r="B235" t="str">
+        <v>RUPSA PRAMANIK</v>
+      </c>
+      <c r="C235" t="str">
+        <v>120250002037047</v>
+      </c>
+      <c r="D235" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236">
+        <v>48</v>
+      </c>
+      <c r="B236" t="str">
+        <v>ARGHADEEP SAMANTA</v>
+      </c>
+      <c r="C236" t="str">
+        <v>120250002037048</v>
+      </c>
+      <c r="D236" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237">
+        <v>49</v>
+      </c>
+      <c r="B237" t="str">
+        <v>MOUMITA SAMANTA</v>
+      </c>
+      <c r="C237" t="str">
+        <v>120250002037049</v>
+      </c>
+      <c r="D237" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E237" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238">
+        <v>50</v>
+      </c>
+      <c r="B238" t="str">
+        <v>SAYAN SAHA</v>
+      </c>
+      <c r="C238" t="str">
+        <v>120250002037050</v>
+      </c>
+      <c r="D238" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E238" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239">
+        <v>51</v>
+      </c>
+      <c r="B239" t="str">
+        <v>ARITRA BANERJEE</v>
+      </c>
+      <c r="C239" t="str">
+        <v>120250002037051</v>
+      </c>
+      <c r="D239" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240">
+        <v>52</v>
+      </c>
+      <c r="B240" t="str">
+        <v>RITWIK BARMAN</v>
+      </c>
+      <c r="C240" t="str">
+        <v>120250002037052</v>
+      </c>
+      <c r="D240" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241">
+        <v>53</v>
+      </c>
+      <c r="B241" t="str">
+        <v>SUSHMITA PRAMANIK</v>
+      </c>
+      <c r="C241" t="str">
+        <v>120250002037053</v>
+      </c>
+      <c r="D241" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E241" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242">
+        <v>54</v>
+      </c>
+      <c r="B242" t="str">
+        <v>PRIYANKA SEN</v>
+      </c>
+      <c r="C242" t="str">
+        <v>120250002037054</v>
+      </c>
+      <c r="D242" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243">
+        <v>55</v>
+      </c>
+      <c r="B243" t="str">
+        <v>NILADRI PAL</v>
+      </c>
+      <c r="C243" t="str">
+        <v>120250002037055</v>
+      </c>
+      <c r="D243" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244">
+        <v>56</v>
+      </c>
+      <c r="B244" t="str">
+        <v>SAGNIK ADHIKARI</v>
+      </c>
+      <c r="C244" t="str">
+        <v>120250002037056</v>
+      </c>
+      <c r="D244" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245">
+        <v>57</v>
+      </c>
+      <c r="B245" t="str">
+        <v>PALLABI PAL</v>
+      </c>
+      <c r="C245" t="str">
+        <v>120250002037057</v>
+      </c>
+      <c r="D245" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246">
+        <v>58</v>
+      </c>
+      <c r="B246" t="str">
+        <v>RUPSA BISWAS</v>
+      </c>
+      <c r="C246" t="str">
+        <v>120250002037058</v>
+      </c>
+      <c r="D246" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247">
+        <v>59</v>
+      </c>
+      <c r="B247" t="str">
+        <v>ISHITA BARMAN</v>
+      </c>
+      <c r="C247" t="str">
+        <v>120250002037059</v>
+      </c>
+      <c r="D247" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248">
+        <v>60</v>
+      </c>
+      <c r="B248" t="str">
+        <v>NILADRI KUMAR</v>
+      </c>
+      <c r="C248" t="str">
+        <v>120250002037060</v>
+      </c>
+      <c r="D248" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249">
+        <v>61</v>
+      </c>
+      <c r="B249" t="str">
+        <v>MADHUMITA DUTTA</v>
+      </c>
+      <c r="C249" t="str">
+        <v>120250002037061</v>
+      </c>
+      <c r="D249" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Sec A</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250">
+        <v>62</v>
+      </c>
+      <c r="B250" t="str">
+        <v>SUSHMITA MAITY</v>
+      </c>
+      <c r="C250" t="str">
+        <v>120250002037062</v>
+      </c>
+      <c r="D250" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Sec A</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E250"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>